<commit_message>
feat(audio): 音频全量接入 + AudioManager BGM 通道 + 全局点击音
P3 音频落地：16 项音效 + 2 首 BGM 全部接入，AudioManager 不再静默降级。

- Assets/Audio/SFX/ 16 个音效（取自素材包，按 TBAudio 的 logicalName 重命名）；Assets/Audio/BGM/ 含 bgm_battle.mp3 与 bgm_select.wav

- bgm_select.wav 由新增的 PlaceholderBgmGenerator 合成：12s / 44.1kHz / 单声道 16bit，频率对齐到 1/loop 网格 + 首尾交叉淡化，可无缝循环（原素材只有一首战斗曲）

- TBAudio 16 → 18 行（+bgm_select / +bgm_battle，loop=1 / is3d=0）；AudioCatalog 0 → 18，ResTable 经 RegisterAudio() 自动登记（282 → 300 条）

AudioManager 新增 BGM 通道：固定 2 个 AudioSource 做交叉淡化 —— 长音不能进音效池，否则会被「顶掉最旧的一个」逻辑误杀；对外 PlayBgm / StopBgm / CurrentBgm。

新增 AudioFadeDriver：只维护 0~1 的淡化系数，绝不直接写 AudioSource.volume。绝对音量统一由 ApplyBgmVolume() = 基准 × 淡化系数 × 主音量 × (静音?0:1) 计算，否则「玩家调音量」会与「正在进行的淡化」互相覆盖。时间用 unscaledDeltaTime，暂停（timeScale=0）时淡化不冻结。

新增 UiClickSfx：由 UIManager.Open 自动挂到每个界面，每 0.4s 重扫 Button（SelectView 每次显示都会重建关卡按钮，旧引用会失效；判等用 Unity 的 == 而不是 List.Contains）。以后新增界面不必写任何点击音代码。
</commit_message>
<xml_diff>
--- a/Luban/Config/Datas/AudioData.xlsx
+++ b/Luban/Config/Datas/AudioData.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1069,6 +1069,70 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="B20" t="n">
+        <v>17</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>选关BGM</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>bgm_select</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F20" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>选关界面循环</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" t="n">
+        <v>18</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>战斗BGM</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>bgm_battle</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F21" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" t="n">
+        <v>1</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>战斗循环</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>